<commit_message>
docs(ST36): refine classical location and redraw cross-section with three transverse traditions
- Identify '銅曰在膝蓋下三寸䯒骨外廉兩筋間陷中' as Heo Im's altered quotation
  of Tongren vol. 2 in 鍼灸經驗方 「訛穴」 (papers.id 1203), not Tongren text
- Separate Tongren vol. 1 '大筋內' (Target 1≡3) from vol. 2 '兩筋間' (Target 2);
  record the (內經) source-label error in 東醫寶鑑; add Tongren 5-fen depth row
- Add the 「訛穴」 / Lee 2008 dissent on the WHO location and a scoring-impact
  table (no rubric step changes; ARI scores unchanged)
- Redraw Figure 4-1: Target 1≡3, Target 2 (TA–EDL septum) and the medial
  Shenghui variant on one section; rebuild KO/EN HTML; add xlsx sheet

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/01_경혈별_해부생리_분석보고서/ST_족양명위경/ST36_족삼리/ST36_족삼리_해부생리_분석데이터.xlsx
+++ b/01_경혈별_해부생리_분석보고서/ST_족양명위경/ST36_족삼리/ST36_족삼리_해부생리_분석데이터.xlsx
@@ -17,9 +17,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LayerA_papers" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="외부검색로그" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="분기추론_TriTarget" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개정이력" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FMA_해부실체" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="초음파_참고" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고전정위_가로3계통" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="개정이력" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FMA_해부실체" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="초음파_참고" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -100,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -110,6 +111,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1140,7 +1144,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>经络通鉴 19편 L253·L449; 通考 L307</t>
+          <t>经络通鉴 19편 L253·L449; 通考 L307; 《铜人》 卷上 胻骨外大筋内(通考 L243·L307 셋째 계통)</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1156,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>王冰 胻外两筋肉分间 / 铜人卷下·圣济 胻外廉两筋间 = 앞정강근(FMA:22532)–긴발가락폄근(FMA:22534) 근간 중격</t>
+          <t>王冰 胻外两筋肉分间 / 铜人卷下·圣济 胻外廉两筋间 = 앞정강근(FMA:22532)–긴발가락폄근(FMA:22534) 근간 중격 / 「訛穴」 銅曰…兩筋間陷中·自骨邊橫量一寸(papers.id 1203)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1172,7 +1176,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>通考 L215·L231 (현행 편)</t>
+          <t>通考 L215·L231 (현행 편); papers.id 1203 p.38</t>
         </is>
       </c>
     </row>
@@ -1358,534 +1362,459 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="45" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>위치</t>
+          <t>계통</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>원래 내용</t>
+          <t>Target</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>바꾼 내용</t>
+          <t>문헌(시대)</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>근거</t>
+          <t>원문</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>해부 위치(추정)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>근거 포인터(내부)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>판정·비고</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>머리말</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>프레임워크 문구, "실측 논문 148편 전수 역색인"</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>v2.7 인용 블록, ARI 표기 / 근거 묶음 수치(38·109·39)로 교체</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>final_ST36.json notation, pack_ST36.md</t>
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>ⓞ 고전 원문</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Target 1≡3</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>《灵枢·本输》·《黄帝明堂经》(한)</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>下陵膝下三寸，胻骨外三里也 / 在膝下三寸，胻外廉</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>정강뼈 바깥 가장자리 쪽(횡향 미특정)</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>通考 08편 L183·L191; 经络通鉴 19편 L253·L449</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>원천</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>1절</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>通鉴 목차 조각, 证治通鉴 冲脉 고증 문단, 通考 목차 조각</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>《灵枢·本输》·《素问·针解》·《明堂》 원문과 출처 행</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>通考 `(上)_321-400.md` L3096~3248; 通鉴 `(上卷)_801-880.md` L3410~3692; 证治通鉴 `_1-80.md` L1242, L2162</t>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>③ 대근내(大筋内)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Target 1≡3</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>《铜人腧穴针灸图经》 卷上(송)</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>在膝下三寸，胻骨外大筋内宛宛中(2:23)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>앞정강근 근복(《通考》 셋째 계통 = 현대 정위)</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>穴位通鉴 19편 L2166; 通考 08편 L243·L307</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>《铜人》 한 책 안의 첫째 정위</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2절</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>제목뿐인 템플릿</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>시대별 원천/재인용 표</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>같은 원전</t>
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>③ 대근내(大筋内)</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Target 1≡3</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>《神应经》(명)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>在膝盖下三寸，胻骨间大筋内，坐而取之</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>앞정강근 근복</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>穴位通鉴 19편 L2180; 通考 08편 L255</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>'膝盖下' — 王執中 '너무 높음' 경고 대상</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>3절</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>"검증된 고전 이명: -"</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>三里·下陵·鬼邪·下三里 표</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>KJH xlsx 행 122; 通考 L3096~3146; 通鉴 L3412~3428</t>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>③ 대근내(大筋内)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Target 1≡3</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>《東醫寶鑑》 鍼灸篇(조선, 1613)</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>在膝下三寸䯒骨外大筋內宛宛中(銅人)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>앞정강근 근복</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>G:/내 드라이브/도서 번역/01_도서_번역_및_원전/동의보감/동의보감_111_鍼灸篇_鍼灸.md L395</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>卷上을 인용</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>4절</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>범용 Layer 경계 2.5/6.5/16.5/22mm, 'Layer 5 관절낭'</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>ST36 구조 순서(앞정강근→깊은종아리신경·앞정강동정맥→뼈사이막), X·Y 기술, mm 경계는 실측 없음으로 미기재</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>교재 데이터셋; 通考 L3114~3116</t>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>① 양근간(兩筋間)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Target 2</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>王冰 《素问》 주(당)</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>在膝下三寸，胻外两筋肉分间。极重按之，则足跗上动脉止矣</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>TA–EDL 근간 중격</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>穴位通鉴 19편 L2158; 通考 08편 L215; 经络通鉴 1편 L2015~2017</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>촉진 표현의 원천. 동맥 압박 소견</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>5절</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>공식 설명만</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>문헌별 푼수→mm 계산표</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>자침깊이 xlsx 행 121; 通鉴 L3676~3692</t>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>① 양근간(兩筋間)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Target 2</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>《铜人腧穴针灸图经》 卷下(송)</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>在膝下三寸，胻外廉两筋间，当举足取之 / 可灸三壮，针入五分(5:72)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>TA–EDL 근간 중격</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>穴位通鉴 19편 L2168; 通考 08편 L231·L773</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>《铜人》 한 책 안의 둘째 정위. 5푼=11.5mm(Target 2 심도 상한)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>6절</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>"2대 교재 일치" 일반문</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>실제 구조명, 피부신경 차이 명시</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>공통교재 refine.xlsx 상세 행 650~655; 김재효 xlsx 상세 행 954~959</t>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>① 양근간(兩筋間)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Target 2</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>《圣济总录》·《针灸资生经》(송)</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>在膝下三寸胻外廉两筋间，当举足取之 / 犊鼻之下三寸方是三里</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>TA–EDL 근간 중격</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>穴位通鉴 19편 L2106·L2170</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>卷下 계통 재인용; 종향 교감</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>7절</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>규칙 설명만</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>횡향 3계통 표, Δ ≤ 15mm 분기 불요</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>通考 L3190~3248</t>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>① 양근간(兩筋間)</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>Target 2</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>《東醫寶鑑》 鍼灸篇(조선, 1613)</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>在膝下三寸陷中䯒骨外廉兩筋肉分間(內經) … 深則足趺陽脉不見 按之大衝脉不動是正穴</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>TA–EDL 근간 중격</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>동의보감_111_鍼灸篇_鍼灸.md L395</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>출처 표지 오류: 王冰 주를 (內經)으로 표지</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>8절 ①</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>papers.id 5·12·19·27·38·46·54·59(PMID 공란)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>ST36 연구 15편, PMID/DOI 기재</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>pack_ST36.md, 마스터DB.json</t>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>① 양근간(兩筋間)</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Target 2</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>허임 《鍼灸經驗方》 「訛穴」(조선, 1644)</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>銅曰在膝蓋下三寸䯒骨外廉兩筋間陷中 … 自骨邊橫量一寸 該的兩筋間陷中 以手按兩筋間 則足跗上太衝脈不動 … 而俗徒取䯒外廉陷中</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>TA–EDL 근간 중격(뼈 가장자리에서 약 1촌, 촉진으로 확정)</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>papers.id 1203 (이연희 2008, 경락경혈학회지 25(4):31–47) p.38·p.44·p.46; G:/내 드라이브/학습자료/실험 및 연구 논문/2008_경락경혈학회지_이연희_…pdf</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="inlineStr">
+        <is>
+          <t>사용자 제시 문구의 원출처. 《铜人》 원문 아님(卷下 개변 인용). 속간 '䯒外廉陷中'을 오류로 지적; 이연희 2008은 WHO 'on TA'를 같은 오류로 봄</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>8절 ②</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>②=2(B3-01 Head zone 근거)</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>②=1(L4~S1 vs T6~T9 분절 불일치, 상척수 경로)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>final bcheck n=2</t>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>② 내측 편위</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>기록만(Target 제외)</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>《太平圣惠方》(송)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>在膝下三寸，胻骨外大筋内筋骨之间陷者宛宛中</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>정강뼈 가쪽면–앞정강근 사이</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>通考 08편 L199; 穴位通鉴 19편 L2164</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>《通考》 过于偏内侧</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>8절 ②</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>③=1, ④=1(B3-11), ⑤=2</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>③=2, ④=2(B3-12·15·16·17), ⑤=1</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>final bcheck n=3~5</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>8절 ②</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>"부합 판정: 확정"</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>"부합", 동물 한정 표지</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>프레임워크 5절 8번</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>8절 ③</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>없음</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>외부 검색 로그 표</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>pack sync_log</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>9절</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>정의문만</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>$P_{single}$/$P_{comb}$ 실제 분리</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>通考 L3310~3460; 证治通鉴 L1242, L2166</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>10절</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>단일 채점 S_orig 85, ARI-Core 79.0, 민감도 78.3, "엄격하게 검증됨"</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>이중 채점 S_orig 81.25, ARI-Core 77.5 ± 0, 민감도 77.1, 범위 제한 결론</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>final_ST36.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>확인 불가</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>《甲乙经》 심도: DB 10푼 vs 通鉴 인용 "一寸五分"(15푼). 원 《甲乙经》 미대조로 DB값 유지, 이문 병기</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>자침깊이 xlsx 행 121; 通鉴 L3676</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>확인 불가</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>papers.id 1841 DOI가 저널과 불일치 의심. DB 수정은 하지 않음</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>마스터DB.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>인용 제외</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>pack 랜드마크 papers.id 1700</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>서지 검증 불가(superseded)로 미인용, 체성-자율 반사 틀은 B3-04·B3-05로 인용</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>조정자 통지 2026-10-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>구판 점수</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>구판 v2.6 점수 79.0(비교 불가)</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>`_구판_v2.6/` 보고서</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>FMA_해부실체 시트 신설 (2026-10-23)</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>FMA 5.1.0 실체 ID·지배신경·줄기·분절·교재 비교 추가. ARI-Core 77.5 ± 0 (B)·SI 75 불변</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>fma_query.py profile ST36; 보고서 4·6·8절·부록 A</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>초음파_참고 시트·그림 4-2 (2026-10-23)</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>앞정강근 공개 초음파 통계, 1896 TI, Rank 6 재실행 로그. 점수 불변</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Marzola 2021; PMID 42500462</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>2026-10-25 Framework 2.7.7 (문헌스크리닝·ARI_v3.0·분기추론 시트)</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>3대 원전, 단일 Target(T1), Δ ≤ 15mm 분기 불요</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>4대 원전 대조 10행(经络通鉴·证治通鉴 한글번역·通考 현행 편, 파일·행 포인터) 추가; T1→Target 1≡3(점수 불변, ④ 재점검 100 유지); Target 2(王冰 两筋间 근간 중격) 신규 — 10mm 기준으로 T2–T3 분기, 단일 채점(예비) 57.5 (C·H); Tri-Target 좌표·Δ 시트 신설</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Framework 2.7.7; 분기 기준 Δ &gt; 10mm(2026-10-25)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ARI_v3.0·B-Check·분기추론 (2026-10-25 Target 2 이중 채점)</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Target 2 단일 채점(예비) 57.5 (C·H), B-Check 3/12, 분기 판정 예비</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>채점자 B 독립 채점 추가 → Target 2 56.25 ± 1.25 (C·H), 민감도 53.1 (D, 가중치 민감), B-Check 최종 7/12; Target 1≡3 단독 우위 확정</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>정본 Rank 7; 채점자 B(점수 가린 사본 사용)</t>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>현대</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Target 1≡3</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>교재·WHO</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>犊鼻下3寸，胫骨前嵴外一横指，胫骨前肌中</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>앞정강근 근복</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>通考 08편 L295~303·L307</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>이연희 2008 반론 병기</t>
         </is>
       </c>
     </row>
@@ -1895,6 +1824,570 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>위치</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>원래 내용</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>바꾼 내용</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>근거</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>머리말</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>프레임워크 문구, "실측 논문 148편 전수 역색인"</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>v2.7 인용 블록, ARI 표기 / 근거 묶음 수치(38·109·39)로 교체</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>final_ST36.json notation, pack_ST36.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1절</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>通鉴 목차 조각, 证治通鉴 冲脉 고증 문단, 通考 목차 조각</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>《灵枢·本输》·《素问·针解》·《明堂》 원문과 출처 행</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>通考 `(上)_321-400.md` L3096~3248; 通鉴 `(上卷)_801-880.md` L3410~3692; 证治通鉴 `_1-80.md` L1242, L2162</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2절</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>제목뿐인 템플릿</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>시대별 원천/재인용 표</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>같은 원전</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3절</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>"검증된 고전 이명: -"</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>三里·下陵·鬼邪·下三里 표</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>KJH xlsx 행 122; 通考 L3096~3146; 通鉴 L3412~3428</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4절</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>범용 Layer 경계 2.5/6.5/16.5/22mm, 'Layer 5 관절낭'</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ST36 구조 순서(앞정강근→깊은종아리신경·앞정강동정맥→뼈사이막), X·Y 기술, mm 경계는 실측 없음으로 미기재</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>교재 데이터셋; 通考 L3114~3116</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5절</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>공식 설명만</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>문헌별 푼수→mm 계산표</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>자침깊이 xlsx 행 121; 通鉴 L3676~3692</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>6절</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>"2대 교재 일치" 일반문</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>실제 구조명, 피부신경 차이 명시</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>공통교재 refine.xlsx 상세 행 650~655; 김재효 xlsx 상세 행 954~959</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>7절</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>규칙 설명만</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>횡향 3계통 표, Δ ≤ 15mm 분기 불요</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>通考 L3190~3248</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>8절 ①</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>papers.id 5·12·19·27·38·46·54·59(PMID 공란)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ST36 연구 15편, PMID/DOI 기재</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>pack_ST36.md, 마스터DB.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>8절 ②</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>②=2(B3-01 Head zone 근거)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>②=1(L4~S1 vs T6~T9 분절 불일치, 상척수 경로)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>final bcheck n=2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8절 ②</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>③=1, ④=1(B3-11), ⑤=2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>③=2, ④=2(B3-12·15·16·17), ⑤=1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>final bcheck n=3~5</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>8절 ②</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>"부합 판정: 확정"</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>"부합", 동물 한정 표지</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>프레임워크 5절 8번</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>8절 ③</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>외부 검색 로그 표</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>pack sync_log</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>9절</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>정의문만</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>$P_{single}$/$P_{comb}$ 실제 분리</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>通考 L3310~3460; 证治通鉴 L1242, L2166</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10절</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>단일 채점 S_orig 85, ARI-Core 79.0, 민감도 78.3, "엄격하게 검증됨"</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>이중 채점 S_orig 81.25, ARI-Core 77.5 ± 0, 민감도 77.1, 범위 제한 결론</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>final_ST36.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>확인 불가</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>《甲乙经》 심도: DB 10푼 vs 通鉴 인용 "一寸五分"(15푼). 원 《甲乙经》 미대조로 DB값 유지, 이문 병기</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>자침깊이 xlsx 행 121; 通鉴 L3676</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>확인 불가</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>papers.id 1841 DOI가 저널과 불일치 의심. DB 수정은 하지 않음</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>마스터DB.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>인용 제외</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>pack 랜드마크 papers.id 1700</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>서지 검증 불가(superseded)로 미인용, 체성-자율 반사 틀은 B3-04·B3-05로 인용</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>조정자 통지 2026-10-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>구판 점수</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>구판 v2.6 점수 79.0(비교 불가)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>`_구판_v2.6/` 보고서</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>FMA_해부실체 시트 신설 (2026-10-23)</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>FMA 5.1.0 실체 ID·지배신경·줄기·분절·교재 비교 추가. ARI-Core 77.5 ± 0 (B)·SI 75 불변</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>fma_query.py profile ST36; 보고서 4·6·8절·부록 A</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>초음파_참고 시트·그림 4-2 (2026-10-23)</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>앞정강근 공개 초음파 통계, 1896 TI, Rank 6 재실행 로그. 점수 불변</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Marzola 2021; PMID 42500462</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-25 Framework 2.7.7 (문헌스크리닝·ARI_v3.0·분기추론 시트)</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>3대 원전, 단일 Target(T1), Δ ≤ 15mm 분기 불요</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>4대 원전 대조 10행(经络通鉴·证治通鉴 한글번역·通考 현행 편, 파일·행 포인터) 추가; T1→Target 1≡3(점수 불변, ④ 재점검 100 유지); Target 2(王冰 两筋间 근간 중격) 신규 — 10mm 기준으로 T2–T3 분기, 단일 채점(예비) 57.5 (C·H); Tri-Target 좌표·Δ 시트 신설</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Framework 2.7.7; 분기 기준 Δ &gt; 10mm(2026-10-25)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ARI_v3.0·B-Check·분기추론 (2026-10-25 Target 2 이중 채점)</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Target 2 단일 채점(예비) 57.5 (C·H), B-Check 3/12, 분기 판정 예비</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>채점자 B 독립 채점 추가 → Target 2 56.25 ± 1.25 (C·H), 민감도 53.1 (D, 가중치 민감), B-Check 최종 7/12; Target 1≡3 단독 우위 확정</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>정본 Rank 7; 채점자 B(점수 가린 사본 사용)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-26 고전 정위 정밀화 (고전정위_가로3계통 시트 신설·분기추론 보강)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>《铜人》 卷上·卷下 미분리, "銅曰…兩筋間陷中" 출처 미확인, 그림 4-1 단일 경로</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>'銅曰…' = 허임 《鍼灸經驗方》 「訛穴」의 《铜人》 卷下 개변 인용으로 판별; 《铜人》 卷上(Target 1≡3)·卷下(Target 2) 분리; 《東醫寶鑑》 (內經) 표지 오류 기록; 그림 4-1 가로 3계통 개정. ARI 점수 불변</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>papers.id 1203 p.38·44·46; 穴位通鉴 19편 L2166~2180; 通考 08편 L231~255·L307·L773; 经络通鉴 1편 L2015~2017; 동의보감 鍼灸篇</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2353,7 +2846,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>